<commit_message>
new notification of the dgft and gst notification
</commit_message>
<xml_diff>
--- a/backend/PDF_DOC/GST/Instruction And Guidelines/Instruction And Guidelines.xlsx
+++ b/backend/PDF_DOC/GST/Instruction And Guidelines/Instruction And Guidelines.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A587FEB2-CBF0-40F3-BD15-2BFAB357D3E7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1039C659-CC63-4960-8995-73284FE0C87D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
   <si>
     <t>Number</t>
   </si>
@@ -112,6 +112,12 @@
   </si>
   <si>
     <t>Instructions and Guidelines : 2026</t>
+  </si>
+  <si>
+    <t>Instruction No. 01/2026-GST</t>
+  </si>
+  <si>
+    <t>Instruction regarding Coordination with State Mining Authorities for sharing information relating to illegal mining and transportation of minerals.</t>
   </si>
 </sst>
 </file>
@@ -454,12 +460,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="19.140625" customWidth="1"/>
-    <col min="3" max="3" width="99" customWidth="1"/>
+    <col min="3" max="3" width="132.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
@@ -476,6 +482,17 @@
       </c>
       <c r="C4" s="3" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="2">
+        <v>46237</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>